<commit_message>
Implemented changes in indicator names (letnica), updated market charts
</commit_message>
<xml_diff>
--- a/data/Sezonskost prenocitev po mesecih in trgih - 2024.xlsx
+++ b/data/Sezonskost prenocitev po mesecih in trgih - 2024.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/peter/Desktop/Slovenija/Razširjeni kazalniki/streamlit app/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32C0BB60-88FE-E549-AB5A-6AFDBEC7BC3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{383FBA9A-2438-6D48-A486-2C96B5A14326}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3700" yWindow="740" windowWidth="39060" windowHeight="41200" activeTab="4" xr2:uid="{78CD7F91-F634-084B-8E20-116EB340D257}"/>
+    <workbookView xWindow="3700" yWindow="740" windowWidth="39060" windowHeight="41200" activeTab="1" xr2:uid="{78CD7F91-F634-084B-8E20-116EB340D257}"/>
   </bookViews>
   <sheets>
     <sheet name="Občine" sheetId="1" r:id="rId1"/>
@@ -753,9 +753,6 @@
     <t>Julijske Alpe</t>
   </si>
   <si>
-    <t>Gorenjska</t>
-  </si>
-  <si>
     <t>Goriško, Vipava, Kras</t>
   </si>
   <si>
@@ -880,6 +877,9 @@
   </si>
   <si>
     <t>Termalna panonska Slovenija</t>
+  </si>
+  <si>
+    <t>Predalpska Slovenija (vzh.Gorenjska)</t>
   </si>
 </sst>
 </file>
@@ -71948,7 +71948,7 @@
     </row>
     <row r="2" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B2" t="s">
         <v>214</v>
@@ -72935,7 +72935,7 @@
     </row>
     <row r="5" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>237</v>
+        <v>279</v>
       </c>
       <c r="B5">
         <v>26914</v>
@@ -73264,7 +73264,7 @@
     </row>
     <row r="6" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B6">
         <v>24840</v>
@@ -73593,7 +73593,7 @@
     </row>
     <row r="7" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B7">
         <v>82556</v>
@@ -73922,7 +73922,7 @@
     </row>
     <row r="8" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B8">
         <v>27422</v>
@@ -74251,7 +74251,7 @@
     </row>
     <row r="9" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B9">
         <v>118060</v>
@@ -74580,7 +74580,7 @@
     </row>
     <row r="10" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B10">
         <v>107176</v>
@@ -74909,7 +74909,7 @@
     </row>
     <row r="11" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B11">
         <v>31105</v>
@@ -75238,7 +75238,7 @@
     </row>
     <row r="12" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B12">
         <v>56738</v>
@@ -75567,7 +75567,7 @@
     </row>
     <row r="13" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B13">
         <v>39026</v>
@@ -76048,7 +76048,7 @@
     </row>
     <row r="2" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B2" t="s">
         <v>214</v>
@@ -76377,7 +76377,7 @@
     </row>
     <row r="3" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B3">
         <v>466</v>
@@ -76706,7 +76706,7 @@
     </row>
     <row r="4" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B4">
         <v>2526</v>
@@ -78351,7 +78351,7 @@
     </row>
     <row r="9" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B9">
         <v>7922</v>
@@ -79009,7 +79009,7 @@
     </row>
     <row r="11" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B11">
         <v>39026</v>
@@ -79667,7 +79667,7 @@
     </row>
     <row r="13" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B13">
         <v>22425</v>
@@ -79996,7 +79996,7 @@
     </row>
     <row r="14" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B14">
         <v>6463</v>
@@ -80654,7 +80654,7 @@
     </row>
     <row r="16" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B16">
         <v>4161</v>
@@ -81312,7 +81312,7 @@
     </row>
     <row r="18" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B18">
         <v>2358</v>
@@ -81641,7 +81641,7 @@
     </row>
     <row r="19" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B19">
         <v>7810</v>
@@ -81970,7 +81970,7 @@
     </row>
     <row r="20" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B20">
         <v>21616</v>
@@ -82957,7 +82957,7 @@
     </row>
     <row r="23" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B23">
         <v>6164</v>
@@ -83944,7 +83944,7 @@
     </row>
     <row r="26" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B26">
         <v>57657</v>
@@ -84273,7 +84273,7 @@
     </row>
     <row r="27" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B27">
         <v>13021</v>
@@ -84931,7 +84931,7 @@
     </row>
     <row r="29" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B29">
         <v>56738</v>
@@ -85260,7 +85260,7 @@
     </row>
     <row r="30" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B30">
         <v>44720</v>
@@ -86576,7 +86576,7 @@
     </row>
     <row r="34" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B34">
         <v>41581</v>
@@ -87234,7 +87234,7 @@
     </row>
     <row r="36" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B36">
         <v>5955</v>
@@ -87563,7 +87563,7 @@
     </row>
     <row r="37" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B37">
         <v>5029</v>
@@ -87892,7 +87892,7 @@
     </row>
     <row r="38" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B38">
         <v>3534</v>
@@ -88373,7 +88373,7 @@
     </row>
     <row r="2" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B2" t="s">
         <v>214</v>
@@ -88702,7 +88702,7 @@
     </row>
     <row r="3" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B3">
         <v>1082</v>
@@ -89031,7 +89031,7 @@
     </row>
     <row r="4" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B4">
         <v>3328</v>
@@ -89360,7 +89360,7 @@
     </row>
     <row r="5" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B5">
         <v>1260</v>
@@ -89689,7 +89689,7 @@
     </row>
     <row r="6" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B6">
         <v>113</v>
@@ -90018,7 +90018,7 @@
     </row>
     <row r="7" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B7">
         <v>332</v>
@@ -90347,7 +90347,7 @@
     </row>
     <row r="8" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B8">
         <v>452</v>
@@ -90676,7 +90676,7 @@
     </row>
     <row r="9" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B9">
         <v>929</v>
@@ -91005,7 +91005,7 @@
     </row>
     <row r="10" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B10">
         <v>2698</v>
@@ -91486,7 +91486,7 @@
     </row>
     <row r="2" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B2" t="s">
         <v>214</v>
@@ -91815,7 +91815,7 @@
     </row>
     <row r="3" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B3">
         <v>312388</v>
@@ -92144,7 +92144,7 @@
     </row>
     <row r="4" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B4">
         <v>81997</v>
@@ -92473,7 +92473,7 @@
     </row>
     <row r="5" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B5">
         <v>135606</v>
@@ -92802,7 +92802,7 @@
     </row>
     <row r="6" spans="1:109" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B6">
         <v>216435</v>

</xml_diff>